<commit_message>
Referat 2 jetzt Neutral
</commit_message>
<xml_diff>
--- a/besetzung.xlsx
+++ b/besetzung.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://thaddenschulede-my.sharepoint.com/personal/lepold_thaddenschule_de/Documents/09 Musik/2025 Elisabeth/alt/Webseite/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git\thadden27\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11" documentId="8_{3028552A-8752-4668-BCF5-26AD18D9605D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{17F97B5E-C7A0-4DB4-87A7-31812DE717BB}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F445666-B333-4F32-AB79-C799E16CBA4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="16440" windowHeight="28320" xr2:uid="{870A77A3-6497-424F-BFDB-56D4CBDBF5BF}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{870A77A3-6497-424F-BFDB-56D4CBDBF5BF}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -137,9 +137,6 @@
     <t>3.3</t>
   </si>
   <si>
-    <t>3.4</t>
-  </si>
-  <si>
     <t>Schauspiel</t>
   </si>
   <si>
@@ -332,7 +329,10 @@
     <t> Eine Heldin A</t>
   </si>
   <si>
-    <t> Eine Heldin B</t>
+    <t>12.3</t>
+  </si>
+  <si>
+    <t>Kann Schule neutral sein?</t>
   </si>
 </sst>
 </file>
@@ -450,7 +450,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="16" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
@@ -476,6 +476,7 @@
     <xf numFmtId="16" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -811,22 +812,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7EAA9A49-82B2-433C-BF39-5078DFD427BF}">
   <dimension ref="A1:O41"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="38.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.85546875" style="9" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="38.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.88671875" style="9" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="6" style="10" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.140625" style="9" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="19.5703125" style="10" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="19.5703125" style="9" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.109375" style="9" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="19.5546875" style="10" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="19.5546875" style="9" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -840,10 +841,10 @@
         <v>27</v>
       </c>
       <c r="E1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G1" s="5" t="s">
         <v>2</v>
@@ -873,7 +874,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>12</v>
       </c>
@@ -887,7 +888,7 @@
       <c r="G2" s="7"/>
       <c r="O2" s="7"/>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>13</v>
       </c>
@@ -898,13 +899,13 @@
         <v>21</v>
       </c>
       <c r="F3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="N3" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>17</v>
       </c>
@@ -918,7 +919,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>18</v>
       </c>
@@ -929,7 +930,7 @@
         <v>21</v>
       </c>
       <c r="F5" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I5" t="s">
         <v>21</v>
@@ -938,7 +939,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>19</v>
       </c>
@@ -949,7 +950,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>22</v>
       </c>
@@ -964,7 +965,7 @@
       </c>
       <c r="E7" s="2"/>
       <c r="F7" s="2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="G7" s="7"/>
       <c r="J7" s="8"/>
@@ -973,12 +974,12 @@
       </c>
       <c r="O7" s="7"/>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
+        <v>69</v>
+      </c>
+      <c r="B8" s="21" t="s">
         <v>70</v>
-      </c>
-      <c r="B8" s="21" t="s">
-        <v>71</v>
       </c>
       <c r="C8" s="22" t="s">
         <v>21</v>
@@ -988,7 +989,7 @@
       </c>
       <c r="E8" s="21"/>
       <c r="F8" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G8" s="9" t="s">
         <v>21</v>
@@ -1009,7 +1010,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:15" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>24</v>
       </c>
@@ -1026,7 +1027,7 @@
       <c r="J9" s="17"/>
       <c r="O9" s="16"/>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>28</v>
       </c>
@@ -1037,15 +1038,15 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>29</v>
       </c>
       <c r="B11" s="24" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F11" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="G11" s="9" t="s">
         <v>21</v>
@@ -1060,7 +1061,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>32</v>
       </c>
@@ -1071,89 +1072,82 @@
         <v>21</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>33</v>
-      </c>
-      <c r="B13" s="24" t="s">
-        <v>98</v>
-      </c>
-      <c r="F13" t="s">
+    <row r="13" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C13" s="7"/>
+      <c r="D13" s="8"/>
+      <c r="G13" s="7"/>
+      <c r="J13" s="8"/>
+      <c r="O13" s="7"/>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>37</v>
+      </c>
+      <c r="B14" t="s">
+        <v>36</v>
+      </c>
+      <c r="C14" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="F14" t="s">
         <v>93</v>
       </c>
-      <c r="G13" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="L13" t="s">
-        <v>21</v>
-      </c>
-      <c r="M13" t="s">
-        <v>21</v>
-      </c>
-      <c r="N13" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="14" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="C14" s="7"/>
-      <c r="D14" s="8"/>
-      <c r="G14" s="7"/>
-      <c r="J14" s="8"/>
-      <c r="O14" s="7"/>
-    </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="J14" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="O14" s="9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>38</v>
       </c>
       <c r="B15" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C15" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="F15" t="s">
-        <v>94</v>
-      </c>
-      <c r="J15" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="O15" s="9" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>39</v>
-      </c>
-      <c r="B16" t="s">
-        <v>40</v>
-      </c>
-      <c r="C16" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="E16" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="17" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="E15" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="D16" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G16" s="7"/>
+      <c r="J16" s="8"/>
+      <c r="O16" s="7"/>
+    </row>
+    <row r="17" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="C17" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="D17" s="8" t="s">
-        <v>21</v>
-      </c>
+      <c r="C17" s="7"/>
+      <c r="D17" s="8"/>
       <c r="E17" s="1" t="s">
         <v>21</v>
       </c>
@@ -1161,43 +1155,41 @@
       <c r="J17" s="8"/>
       <c r="O17" s="7"/>
     </row>
-    <row r="18" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
-        <v>86</v>
+        <v>40</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="C18" s="7"/>
+        <v>41</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>21</v>
+      </c>
       <c r="D18" s="8"/>
-      <c r="E18" s="1" t="s">
-        <v>21</v>
-      </c>
       <c r="G18" s="7"/>
       <c r="J18" s="8"/>
       <c r="O18" s="7"/>
     </row>
-    <row r="19" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="B19" s="1" t="s">
+    <row r="19" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
         <v>42</v>
       </c>
-      <c r="C19" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="D19" s="8"/>
-      <c r="G19" s="7"/>
-      <c r="J19" s="8"/>
-      <c r="O19" s="7"/>
-    </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="B19" t="s">
+        <v>43</v>
+      </c>
+      <c r="C19" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="E19" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B20" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C20" s="9" t="s">
         <v>21</v>
@@ -1205,168 +1197,187 @@
       <c r="E20" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>45</v>
-      </c>
-      <c r="B21" t="s">
+      <c r="F20" t="s">
+        <v>94</v>
+      </c>
+      <c r="L20" t="s">
+        <v>21</v>
+      </c>
+      <c r="M20" t="s">
+        <v>21</v>
+      </c>
+      <c r="N20" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" s="18" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="18" t="s">
         <v>46</v>
       </c>
-      <c r="C21" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="E21" t="s">
-        <v>21</v>
-      </c>
-      <c r="F21" t="s">
+      <c r="C21" s="19"/>
+      <c r="D21" s="20"/>
+      <c r="G21" s="19"/>
+      <c r="J21" s="20"/>
+      <c r="O21" s="19"/>
+    </row>
+    <row r="22" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C22" s="7"/>
+      <c r="D22" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="G22" s="7"/>
+      <c r="J22" s="8"/>
+      <c r="O22" s="7"/>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>49</v>
+      </c>
+      <c r="B23" t="s">
+        <v>50</v>
+      </c>
+      <c r="D23" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="E23" t="s">
+        <v>21</v>
+      </c>
+      <c r="F23" t="s">
+        <v>94</v>
+      </c>
+      <c r="M23" t="s">
+        <v>21</v>
+      </c>
+      <c r="O23" s="9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>51</v>
+      </c>
+      <c r="B24" t="s">
+        <v>52</v>
+      </c>
+      <c r="D24" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="E24" t="s">
+        <v>21</v>
+      </c>
+      <c r="F24" t="s">
+        <v>94</v>
+      </c>
+      <c r="H24" t="s">
+        <v>21</v>
+      </c>
+      <c r="K24" t="s">
+        <v>21</v>
+      </c>
+      <c r="M24" t="s">
+        <v>21</v>
+      </c>
+      <c r="O24" s="9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>53</v>
+      </c>
+      <c r="B25" t="s">
+        <v>54</v>
+      </c>
+      <c r="D25" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="E25" t="s">
+        <v>21</v>
+      </c>
+      <c r="F25" t="s">
+        <v>92</v>
+      </c>
+      <c r="K25" t="s">
+        <v>21</v>
+      </c>
+      <c r="O25" s="9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>55</v>
+      </c>
+      <c r="B26" t="s">
+        <v>56</v>
+      </c>
+      <c r="D26" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="E26" t="s">
+        <v>21</v>
+      </c>
+      <c r="F26" t="s">
+        <v>92</v>
+      </c>
+      <c r="H26" t="s">
+        <v>21</v>
+      </c>
+      <c r="K26" t="s">
+        <v>21</v>
+      </c>
+      <c r="M26" t="s">
+        <v>21</v>
+      </c>
+      <c r="O26" s="9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="27" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C27" s="7"/>
+      <c r="D27" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F27" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="L21" t="s">
-        <v>21</v>
-      </c>
-      <c r="M21" t="s">
-        <v>21</v>
-      </c>
-      <c r="N21" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="22" spans="1:15" s="18" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="18" t="s">
-        <v>47</v>
-      </c>
-      <c r="C22" s="19"/>
-      <c r="D22" s="20"/>
-      <c r="G22" s="19"/>
-      <c r="J22" s="20"/>
-      <c r="O22" s="19"/>
-    </row>
-    <row r="23" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="C23" s="7"/>
-      <c r="D23" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="G23" s="7"/>
-      <c r="J23" s="8"/>
-      <c r="O23" s="7"/>
-    </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>50</v>
-      </c>
-      <c r="B24" t="s">
-        <v>51</v>
-      </c>
-      <c r="D24" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="E24" t="s">
-        <v>21</v>
-      </c>
-      <c r="F24" t="s">
-        <v>95</v>
-      </c>
-      <c r="M24" t="s">
-        <v>21</v>
-      </c>
-      <c r="O24" s="9" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>52</v>
-      </c>
-      <c r="B25" t="s">
-        <v>53</v>
-      </c>
-      <c r="D25" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="E25" t="s">
-        <v>21</v>
-      </c>
-      <c r="F25" t="s">
-        <v>95</v>
-      </c>
-      <c r="H25" t="s">
-        <v>21</v>
-      </c>
-      <c r="K25" t="s">
-        <v>21</v>
-      </c>
-      <c r="M25" t="s">
-        <v>21</v>
-      </c>
-      <c r="O25" s="9" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>54</v>
-      </c>
-      <c r="B26" t="s">
-        <v>55</v>
-      </c>
-      <c r="D26" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="E26" t="s">
-        <v>21</v>
-      </c>
-      <c r="F26" t="s">
-        <v>93</v>
-      </c>
-      <c r="K26" t="s">
-        <v>21</v>
-      </c>
-      <c r="O26" s="9" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>56</v>
-      </c>
-      <c r="B27" t="s">
-        <v>57</v>
-      </c>
-      <c r="D27" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="E27" t="s">
-        <v>21</v>
-      </c>
-      <c r="F27" t="s">
-        <v>93</v>
-      </c>
-      <c r="H27" t="s">
-        <v>21</v>
-      </c>
-      <c r="K27" t="s">
-        <v>21</v>
-      </c>
-      <c r="M27" t="s">
-        <v>21</v>
-      </c>
-      <c r="O27" s="9" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="28" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="G27" s="7"/>
+      <c r="I27" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="J27" s="8"/>
+      <c r="L27" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="M27" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="N27" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="O27" s="7"/>
+    </row>
+    <row r="28" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C28" s="7"/>
       <c r="D28" s="8" t="s">
@@ -1375,36 +1386,21 @@
       <c r="E28" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="F28" s="1" t="s">
-        <v>96</v>
-      </c>
       <c r="G28" s="7"/>
-      <c r="I28" s="1" t="s">
-        <v>21</v>
-      </c>
       <c r="J28" s="8"/>
-      <c r="L28" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="M28" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="N28" s="1" t="s">
-        <v>21</v>
-      </c>
       <c r="O28" s="7"/>
     </row>
-    <row r="29" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="C29" s="7"/>
-      <c r="D29" s="8" t="s">
-        <v>21</v>
-      </c>
+        <v>62</v>
+      </c>
+      <c r="C29" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="D29" s="8"/>
       <c r="E29" s="1" t="s">
         <v>21</v>
       </c>
@@ -1412,62 +1408,67 @@
       <c r="J29" s="8"/>
       <c r="O29" s="7"/>
     </row>
-    <row r="30" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="C30" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="D30" s="8"/>
-      <c r="E30" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C30" s="7"/>
+      <c r="D30" s="8" t="s">
         <v>21</v>
       </c>
       <c r="G30" s="7"/>
       <c r="J30" s="8"/>
       <c r="O30" s="7"/>
     </row>
-    <row r="31" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="B31" s="1" t="s">
+    <row r="31" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
         <v>65</v>
       </c>
-      <c r="C31" s="7"/>
-      <c r="D31" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="G31" s="7"/>
-      <c r="J31" s="8"/>
-      <c r="O31" s="7"/>
-    </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="B31" t="s">
+        <v>67</v>
+      </c>
+      <c r="D31" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="32" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>66</v>
       </c>
-      <c r="B32" t="s">
+      <c r="B32" s="24" t="s">
+        <v>98</v>
+      </c>
+      <c r="F32" t="s">
+        <v>92</v>
+      </c>
+      <c r="G32" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="L32" t="s">
+        <v>21</v>
+      </c>
+      <c r="M32" t="s">
+        <v>21</v>
+      </c>
+      <c r="N32" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="33" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A33" s="25" t="s">
+        <v>97</v>
+      </c>
+      <c r="B33" t="s">
         <v>68</v>
       </c>
-      <c r="D32" s="10" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>67</v>
-      </c>
-      <c r="B33" t="s">
-        <v>69</v>
-      </c>
       <c r="D33" s="10" t="s">
         <v>21</v>
       </c>
       <c r="F33" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="G33" s="9" t="s">
         <v>21</v>
@@ -1491,12 +1492,12 @@
         <v>21</v>
       </c>
     </row>
-    <row r="34" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A34" s="1">
         <v>13</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C34" s="7" t="s">
         <v>21</v>
@@ -1508,57 +1509,57 @@
       <c r="J34" s="8"/>
       <c r="O34" s="7"/>
     </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
+        <v>78</v>
+      </c>
+      <c r="B35" t="s">
+        <v>72</v>
+      </c>
+      <c r="C35" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="E35" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="36" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>77</v>
+      </c>
+      <c r="B36" t="s">
         <v>79</v>
       </c>
-      <c r="B35" t="s">
+      <c r="F36" t="s">
+        <v>91</v>
+      </c>
+      <c r="G36" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="H36" t="s">
+        <v>21</v>
+      </c>
+      <c r="I36" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="37" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>74</v>
+      </c>
+      <c r="B37" t="s">
         <v>73</v>
       </c>
-      <c r="C35" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="E35" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>78</v>
-      </c>
-      <c r="B36" t="s">
-        <v>80</v>
-      </c>
-      <c r="F36" t="s">
-        <v>92</v>
-      </c>
-      <c r="G36" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="H36" t="s">
-        <v>21</v>
-      </c>
-      <c r="I36" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
+      <c r="D37" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="E37" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="38" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
         <v>75</v>
-      </c>
-      <c r="B37" t="s">
-        <v>74</v>
-      </c>
-      <c r="D37" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="E37" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>76</v>
       </c>
       <c r="B38" t="s">
         <v>20</v>
@@ -1570,7 +1571,7 @@
         <v>21</v>
       </c>
       <c r="F38" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="L38" t="s">
         <v>21</v>
@@ -1582,45 +1583,45 @@
         <v>21</v>
       </c>
     </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B39" t="s">
+        <v>80</v>
+      </c>
+      <c r="D39" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="E39" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="40" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
         <v>81</v>
       </c>
-      <c r="D39" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="E39" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
+      <c r="B40" t="s">
         <v>82</v>
       </c>
-      <c r="B40" t="s">
+      <c r="D40" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="E40" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="41" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="D40" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="E40" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="41" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="1" t="s">
+      <c r="B41" s="1" t="s">
         <v>84</v>
-      </c>
-      <c r="B41" s="1" t="s">
-        <v>85</v>
       </c>
       <c r="C41" s="7"/>
       <c r="D41" s="8"/>
       <c r="F41" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="G41" s="7" t="s">
         <v>21</v>

</xml_diff>

<commit_message>
neu nummern und szene gestrichen
</commit_message>
<xml_diff>
--- a/besetzung.xlsx
+++ b/besetzung.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Thadden27\thadden27\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{961D446E-B326-4352-8077-EDF0B85B8033}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B74584BE-AB6F-4E64-88D7-6F6F27058D51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{870A77A3-6497-424F-BFDB-56D4CBDBF5BF}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="106">
   <si>
     <t>Szene</t>
   </si>
@@ -68,9 +68,6 @@
     <t>Tanz</t>
   </si>
   <si>
-    <t>Schuleröffnung</t>
-  </si>
-  <si>
     <t>1</t>
   </si>
   <si>
@@ -137,9 +134,6 @@
     <t>4</t>
   </si>
   <si>
-    <t xml:space="preserve">Schulinspektion </t>
-  </si>
-  <si>
     <t>7</t>
   </si>
   <si>
@@ -167,21 +161,12 @@
     <t>2nd Walz</t>
   </si>
   <si>
-    <t>8.2</t>
-  </si>
-  <si>
     <t>Mambo</t>
   </si>
   <si>
-    <t>8.3</t>
-  </si>
-  <si>
     <t>Tanzparty</t>
   </si>
   <si>
-    <t>8.4</t>
-  </si>
-  <si>
     <t>Eskalation</t>
   </si>
   <si>
@@ -197,12 +182,6 @@
     <t>12</t>
   </si>
   <si>
-    <t>12.1</t>
-  </si>
-  <si>
-    <t>12.2</t>
-  </si>
-  <si>
     <t>2.1</t>
   </si>
   <si>
@@ -218,18 +197,9 @@
     <t xml:space="preserve">Dystopie </t>
   </si>
   <si>
-    <t>13c</t>
-  </si>
-  <si>
-    <t>13d</t>
-  </si>
-  <si>
     <t>Mögliches Happy End</t>
   </si>
   <si>
-    <t>14</t>
-  </si>
-  <si>
     <t>Finale</t>
   </si>
   <si>
@@ -260,18 +230,12 @@
     <t xml:space="preserve">Boyne </t>
   </si>
   <si>
-    <t>12.3</t>
-  </si>
-  <si>
     <t>Kann Schule neutral sein?</t>
   </si>
   <si>
     <t>6.1</t>
   </si>
   <si>
-    <t>9.1</t>
-  </si>
-  <si>
     <t>Bin ich allein?</t>
   </si>
   <si>
@@ -308,9 +272,6 @@
     <t>Vorbereitung zur Flucht</t>
   </si>
   <si>
-    <t>Musikalischer Übergang</t>
-  </si>
-  <si>
     <t>Innerer Monolog: Ich möchte leben</t>
   </si>
   <si>
@@ -347,19 +308,52 @@
     <t>Mach End o Herr mach Ende</t>
   </si>
   <si>
-    <t>13a.1</t>
-  </si>
-  <si>
-    <t>13a.2</t>
-  </si>
-  <si>
-    <t>13b.1</t>
-  </si>
-  <si>
-    <t>13b.2</t>
-  </si>
-  <si>
-    <t>Nach dem Ball (Verarbeitung der Trennung)</t>
+    <t>Osterfeier</t>
+  </si>
+  <si>
+    <t>Nach dem Ball</t>
+  </si>
+  <si>
+    <t>Gestapo in Tuzingen</t>
+  </si>
+  <si>
+    <t>6.2</t>
+  </si>
+  <si>
+    <t>7.3</t>
+  </si>
+  <si>
+    <t>7.4</t>
+  </si>
+  <si>
+    <t>10.1</t>
+  </si>
+  <si>
+    <t>10.2</t>
+  </si>
+  <si>
+    <t>11.3</t>
+  </si>
+  <si>
+    <t>12a.1</t>
+  </si>
+  <si>
+    <t>12a.2</t>
+  </si>
+  <si>
+    <t>12b.1</t>
+  </si>
+  <si>
+    <t>12b.2</t>
+  </si>
+  <si>
+    <t>12c</t>
+  </si>
+  <si>
+    <t>12d</t>
+  </si>
+  <si>
+    <t>13</t>
   </si>
 </sst>
 </file>
@@ -396,7 +390,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -412,6 +406,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.34998626667073579"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -477,7 +477,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="16" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
@@ -509,6 +509,10 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -841,9 +845,31 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="350" row="1">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{71E547F6-03DB-45A4-8800-2182588C5808}">
+  <we:reference id="WA200010215" version="2.0.0.0" store="Omex" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="WA200010215" version="2.0.0.0" store="WA200010215" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="bps.codex_control.document_id" value="&quot;31676971-55d2-40c7-89c4-ed23e1dc6e0f&quot;"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7EAA9A49-82B2-433C-BF39-5078DFD427BF}">
-  <dimension ref="A1:O46"/>
+  <dimension ref="A1:O44"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.5703125" style="25"/>
@@ -868,19 +894,19 @@
         <v>1</v>
       </c>
       <c r="C1" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="D1" s="6" t="s">
-        <v>26</v>
-      </c>
       <c r="E1" t="s">
-        <v>92</v>
+        <v>79</v>
       </c>
       <c r="F1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G1" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="H1" s="5" t="s">
         <v>2</v>
@@ -909,13 +935,13 @@
     </row>
     <row r="2" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="26" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>10</v>
+        <v>90</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D2" s="8"/>
       <c r="H2" s="7"/>
@@ -924,138 +950,138 @@
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="25" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G3" t="s">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="N3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="25" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="25" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G5" t="s">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="J5" s="10" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="O5" s="9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" s="25" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="7" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="26" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B7" s="2" t="s">
-        <v>22</v>
-      </c>
       <c r="C7" s="11" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E7" s="2"/>
       <c r="F7" s="2"/>
       <c r="G7" s="2" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="H7" s="7"/>
       <c r="J7" s="8"/>
       <c r="K7" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="O7" s="7"/>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="25" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="C8" s="22" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D8" s="23" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E8" s="21"/>
       <c r="F8" s="21"/>
       <c r="G8" t="s">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="I8" s="21" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="J8" s="23" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="L8" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="M8" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="N8" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="9" spans="1:15" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="26" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" s="3" t="s">
         <v>23</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>24</v>
       </c>
       <c r="C9" s="13"/>
       <c r="D9" s="14" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E9" s="3"/>
       <c r="F9" s="3"/>
@@ -1066,68 +1092,68 @@
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="25" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B10" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F10" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="25" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B11" s="24" t="s">
-        <v>79</v>
+        <v>67</v>
       </c>
       <c r="G11" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="H11" s="9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="I11" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="L11" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="M11" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="N11" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" s="25" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B12" t="s">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="F12" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="K12" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="13" spans="1:15" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="26" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>81</v>
+        <v>69</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D13" s="17"/>
       <c r="F13" s="4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H13" s="16"/>
       <c r="J13" s="17"/>
@@ -1135,74 +1161,74 @@
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="25" t="s">
-        <v>82</v>
+        <v>70</v>
       </c>
       <c r="B14" t="s">
-        <v>84</v>
+        <v>72</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G14" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="I14" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" s="25" t="s">
-        <v>83</v>
+        <v>71</v>
       </c>
       <c r="B15" t="s">
-        <v>87</v>
+        <v>75</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F15" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" s="25" t="s">
-        <v>85</v>
+        <v>73</v>
       </c>
       <c r="B16" t="s">
-        <v>86</v>
+        <v>74</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G16" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="H16" s="9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="I16" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="O16" s="9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="17" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="26" t="s">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>88</v>
+        <v>76</v>
       </c>
       <c r="C17" s="7"/>
       <c r="D17" s="8" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H17" s="7"/>
       <c r="J17" s="8"/>
@@ -1210,13 +1236,13 @@
     </row>
     <row r="18" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="26" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>33</v>
+        <v>77</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D18" s="8"/>
       <c r="H18" s="7"/>
@@ -1225,542 +1251,513 @@
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" s="25" t="s">
-        <v>76</v>
+        <v>65</v>
       </c>
       <c r="B19" t="s">
-        <v>90</v>
-      </c>
-      <c r="D19" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="M19" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="20" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="26" t="s">
         <v>34</v>
       </c>
-      <c r="B20" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="C20" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="D20" s="8"/>
-      <c r="H20" s="7"/>
-      <c r="J20" s="8"/>
-      <c r="O20" s="7"/>
-    </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A21" s="25" t="s">
+      <c r="C19" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="F19" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A20" s="25" t="s">
+        <v>93</v>
+      </c>
+      <c r="B20" t="s">
+        <v>78</v>
+      </c>
+      <c r="C20" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="F20" t="s">
+        <v>19</v>
+      </c>
+      <c r="G20" t="s">
+        <v>62</v>
+      </c>
+      <c r="L20" t="s">
+        <v>19</v>
+      </c>
+      <c r="M20" t="s">
+        <v>19</v>
+      </c>
+      <c r="N20" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="27" t="s">
+        <v>36</v>
+      </c>
+      <c r="C21" s="19"/>
+      <c r="D21" s="20"/>
+      <c r="H21" s="19"/>
+      <c r="J21" s="20"/>
+      <c r="O21" s="19"/>
+    </row>
+    <row r="22" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="26" t="s">
+        <v>32</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C22" s="7"/>
+      <c r="D22" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="H22" s="7"/>
+      <c r="J22" s="8"/>
+      <c r="O22" s="7"/>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A23" s="25" t="s">
+        <v>33</v>
+      </c>
+      <c r="B23" t="s">
+        <v>40</v>
+      </c>
+      <c r="D23" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="F23" t="s">
+        <v>19</v>
+      </c>
+      <c r="G23" t="s">
+        <v>62</v>
+      </c>
+      <c r="M23" t="s">
+        <v>19</v>
+      </c>
+      <c r="O23" s="9" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A24" s="25" t="s">
         <v>35</v>
       </c>
-      <c r="B21" t="s">
-        <v>36</v>
-      </c>
-      <c r="C21" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="F21" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A22" s="25" t="s">
-        <v>37</v>
-      </c>
-      <c r="B22" t="s">
-        <v>91</v>
-      </c>
-      <c r="C22" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="F22" t="s">
-        <v>20</v>
-      </c>
-      <c r="G22" t="s">
-        <v>72</v>
-      </c>
-      <c r="L22" t="s">
-        <v>20</v>
-      </c>
-      <c r="M22" t="s">
-        <v>20</v>
-      </c>
-      <c r="N22" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="23" spans="1:15" s="18" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="27" t="s">
-        <v>38</v>
-      </c>
-      <c r="C23" s="19"/>
-      <c r="D23" s="20"/>
-      <c r="H23" s="19"/>
-      <c r="J23" s="20"/>
-      <c r="O23" s="19"/>
-    </row>
-    <row r="24" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="26" t="s">
-        <v>39</v>
-      </c>
-      <c r="B24" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C24" s="7"/>
-      <c r="D24" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="H24" s="7"/>
-      <c r="J24" s="8"/>
-      <c r="O24" s="7"/>
+      <c r="B24" t="s">
+        <v>41</v>
+      </c>
+      <c r="D24" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="F24" t="s">
+        <v>19</v>
+      </c>
+      <c r="G24" t="s">
+        <v>62</v>
+      </c>
+      <c r="I24" t="s">
+        <v>19</v>
+      </c>
+      <c r="K24" t="s">
+        <v>19</v>
+      </c>
+      <c r="M24" t="s">
+        <v>19</v>
+      </c>
+      <c r="O24" s="9" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" s="25" t="s">
-        <v>41</v>
+        <v>94</v>
       </c>
       <c r="B25" t="s">
         <v>42</v>
       </c>
       <c r="D25" s="10" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F25" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G25" t="s">
-        <v>72</v>
-      </c>
-      <c r="M25" t="s">
-        <v>20</v>
+        <v>60</v>
+      </c>
+      <c r="K25" t="s">
+        <v>19</v>
       </c>
       <c r="O25" s="9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A26" s="25" t="s">
+        <v>95</v>
+      </c>
+      <c r="B26" t="s">
         <v>43</v>
       </c>
-      <c r="B26" t="s">
-        <v>44</v>
-      </c>
       <c r="D26" s="10" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F26" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G26" t="s">
-        <v>72</v>
+        <v>60</v>
       </c>
       <c r="I26" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="K26" t="s">
-        <v>20</v>
-      </c>
-      <c r="M26" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="O26" s="9" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A27" s="25" t="s">
-        <v>45</v>
-      </c>
-      <c r="B27" t="s">
-        <v>46</v>
-      </c>
-      <c r="D27" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="F27" t="s">
-        <v>20</v>
-      </c>
-      <c r="G27" t="s">
-        <v>70</v>
-      </c>
-      <c r="K27" t="s">
-        <v>20</v>
-      </c>
-      <c r="O27" s="9" t="s">
-        <v>20</v>
-      </c>
+        <v>19</v>
+      </c>
+    </row>
+    <row r="27" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="26" t="s">
+        <v>37</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C27" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="D27" s="8"/>
+      <c r="F27" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="H27" s="7"/>
+      <c r="J27" s="8"/>
+      <c r="O27" s="7"/>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28" s="25" t="s">
-        <v>47</v>
+        <v>96</v>
       </c>
       <c r="B28" t="s">
-        <v>48</v>
-      </c>
-      <c r="D28" s="10" t="s">
-        <v>20</v>
+        <v>86</v>
+      </c>
+      <c r="C28" s="9" t="s">
+        <v>19</v>
       </c>
       <c r="F28" t="s">
-        <v>20</v>
-      </c>
-      <c r="G28" t="s">
-        <v>70</v>
-      </c>
-      <c r="I28" t="s">
-        <v>20</v>
-      </c>
-      <c r="K28" t="s">
-        <v>20</v>
-      </c>
-      <c r="O28" s="9" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="29" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="26" t="s">
-        <v>49</v>
-      </c>
-      <c r="B29" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="C29" s="7"/>
-      <c r="D29" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="H29" s="7"/>
-      <c r="J29" s="8"/>
-      <c r="O29" s="7"/>
-    </row>
-    <row r="30" spans="1:15" s="28" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="25" t="s">
-        <v>77</v>
-      </c>
-      <c r="B30" t="s">
-        <v>78</v>
-      </c>
-      <c r="C30" s="29"/>
-      <c r="D30" s="30" t="s">
-        <v>20</v>
-      </c>
-      <c r="F30" s="28" t="s">
-        <v>20</v>
-      </c>
-      <c r="G30" t="s">
-        <v>73</v>
-      </c>
-      <c r="H30" s="29"/>
-      <c r="J30" s="30" t="s">
-        <v>20</v>
-      </c>
-      <c r="L30" s="28" t="s">
-        <v>20</v>
-      </c>
-      <c r="O30" s="29"/>
-    </row>
-    <row r="31" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="26" t="s">
-        <v>50</v>
-      </c>
-      <c r="B31" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="M28" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A29" s="25" t="s">
+        <v>97</v>
+      </c>
+      <c r="B29" t="s">
+        <v>85</v>
+      </c>
+      <c r="C29" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="F29" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="30" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="26" t="s">
+        <v>44</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="C30" s="7"/>
+      <c r="D30" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="H30" s="7"/>
+      <c r="J30" s="8"/>
+      <c r="O30" s="7"/>
+    </row>
+    <row r="31" spans="1:15" s="28" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="25" t="s">
+        <v>39</v>
+      </c>
+      <c r="B31" t="s">
+        <v>66</v>
+      </c>
+      <c r="C31" s="29"/>
+      <c r="D31" s="30" t="s">
+        <v>19</v>
+      </c>
+      <c r="F31" s="28" t="s">
+        <v>19</v>
+      </c>
+      <c r="G31" t="s">
+        <v>63</v>
+      </c>
+      <c r="H31" s="29"/>
+      <c r="J31" s="30" t="s">
+        <v>19</v>
+      </c>
+      <c r="L31" s="28" t="s">
+        <v>19</v>
+      </c>
+      <c r="O31" s="29"/>
+    </row>
+    <row r="32" spans="1:15" s="32" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="31" t="s">
+        <v>45</v>
+      </c>
+      <c r="B32" s="32" t="s">
         <v>92</v>
       </c>
-      <c r="C31" s="7"/>
-      <c r="D31" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="E31" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="H31" s="7"/>
-      <c r="J31" s="8"/>
-      <c r="O31" s="7"/>
-    </row>
-    <row r="32" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="26" t="s">
-        <v>51</v>
-      </c>
-      <c r="B32" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="C32" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="D32" s="8"/>
-      <c r="F32" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="H32" s="7"/>
-      <c r="J32" s="8"/>
-      <c r="O32" s="7"/>
-    </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A33" s="25" t="s">
-        <v>96</v>
-      </c>
-      <c r="B33" t="s">
-        <v>99</v>
-      </c>
-      <c r="C33" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="F33" t="s">
-        <v>20</v>
-      </c>
-      <c r="M33" t="s">
-        <v>20</v>
-      </c>
+      <c r="C32" s="33" t="s">
+        <v>19</v>
+      </c>
+      <c r="D32" s="34"/>
+      <c r="F32" s="32" t="s">
+        <v>19</v>
+      </c>
+      <c r="H32" s="33"/>
+      <c r="J32" s="34"/>
+      <c r="O32" s="33"/>
+    </row>
+    <row r="33" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="26" t="s">
+        <v>46</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C33" s="7"/>
+      <c r="D33" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="H33" s="7"/>
+      <c r="J33" s="8"/>
+      <c r="O33" s="7"/>
     </row>
     <row r="34" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A34" s="25" t="s">
-        <v>97</v>
+        <v>83</v>
       </c>
       <c r="B34" t="s">
-        <v>98</v>
-      </c>
-      <c r="C34" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="F34" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="35" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="26" t="s">
-        <v>52</v>
-      </c>
-      <c r="B35" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="C35" s="7"/>
-      <c r="D35" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="H35" s="7"/>
-      <c r="J35" s="8"/>
-      <c r="O35" s="7"/>
+        <v>82</v>
+      </c>
+      <c r="D34" s="10" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="35" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A35" s="25" t="s">
+        <v>84</v>
+      </c>
+      <c r="B35" s="24" t="s">
+        <v>64</v>
+      </c>
+      <c r="G35" t="s">
+        <v>60</v>
+      </c>
+      <c r="H35" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="I35" t="s">
+        <v>19</v>
+      </c>
+      <c r="L35" t="s">
+        <v>19</v>
+      </c>
+      <c r="M35" t="s">
+        <v>19</v>
+      </c>
+      <c r="N35" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="36" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A36" s="25" t="s">
-        <v>53</v>
+        <v>98</v>
       </c>
       <c r="B36" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="D36" s="10" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A37" s="25" t="s">
-        <v>54</v>
-      </c>
-      <c r="B37" s="24" t="s">
-        <v>75</v>
-      </c>
-      <c r="G37" t="s">
-        <v>70</v>
-      </c>
-      <c r="H37" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="I37" t="s">
-        <v>20</v>
-      </c>
-      <c r="L37" t="s">
-        <v>20</v>
-      </c>
-      <c r="M37" t="s">
-        <v>20</v>
-      </c>
-      <c r="N37" t="s">
-        <v>20</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="E36" t="s">
+        <v>19</v>
+      </c>
+      <c r="F36" t="s">
+        <v>19</v>
+      </c>
+      <c r="I36" t="s">
+        <v>19</v>
+      </c>
+      <c r="K36" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="37" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="26" t="s">
+        <v>47</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C37" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="D37" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="H37" s="7"/>
+      <c r="J37" s="8"/>
+      <c r="O37" s="7"/>
     </row>
     <row r="38" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A38" s="25" t="s">
-        <v>74</v>
+        <v>99</v>
       </c>
       <c r="B38" t="s">
+        <v>51</v>
+      </c>
+      <c r="C38" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="F38" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="39" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A39" s="25" t="s">
         <v>100</v>
       </c>
-      <c r="D38" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="E38" t="s">
-        <v>20</v>
-      </c>
-      <c r="F38" t="s">
-        <v>20</v>
-      </c>
-      <c r="I38" t="s">
-        <v>20</v>
-      </c>
-      <c r="K38" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="39" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="26">
-        <v>13</v>
-      </c>
-      <c r="B39" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="C39" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="D39" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="H39" s="7"/>
-      <c r="J39" s="8"/>
-      <c r="O39" s="7"/>
+      <c r="B39" t="s">
+        <v>89</v>
+      </c>
+      <c r="G39" t="s">
+        <v>59</v>
+      </c>
+      <c r="H39" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="I39" t="s">
+        <v>19</v>
+      </c>
+      <c r="J39" s="10" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="40" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A40" s="25" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B40" t="s">
-        <v>58</v>
-      </c>
-      <c r="C40" s="9" t="s">
-        <v>20</v>
+        <v>52</v>
+      </c>
+      <c r="D40" s="10" t="s">
+        <v>19</v>
       </c>
       <c r="F40" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="41" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A41" s="25" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B41" t="s">
-        <v>102</v>
+        <v>18</v>
+      </c>
+      <c r="D41" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="F41" t="s">
+        <v>19</v>
       </c>
       <c r="G41" t="s">
-        <v>69</v>
-      </c>
-      <c r="H41" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="I41" t="s">
-        <v>20</v>
-      </c>
-      <c r="J41" s="10" t="s">
-        <v>20</v>
+        <v>63</v>
+      </c>
+      <c r="L41" t="s">
+        <v>19</v>
+      </c>
+      <c r="M41" t="s">
+        <v>19</v>
+      </c>
+      <c r="N41" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="42" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A42" s="25" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B42" t="s">
-        <v>59</v>
+        <v>88</v>
       </c>
       <c r="D42" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="F42" t="s">
-        <v>20</v>
+        <v>19</v>
+      </c>
+      <c r="E42" t="s">
+        <v>19</v>
+      </c>
+      <c r="M42" t="s">
+        <v>19</v>
+      </c>
+      <c r="N42" t="s">
+        <v>19</v>
+      </c>
+      <c r="O42" s="9" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="43" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A43" s="25" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="B43" t="s">
-        <v>19</v>
+        <v>53</v>
       </c>
       <c r="D43" s="10" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F43" t="s">
-        <v>20</v>
-      </c>
-      <c r="G43" t="s">
-        <v>73</v>
-      </c>
-      <c r="L43" t="s">
-        <v>20</v>
-      </c>
-      <c r="M43" t="s">
-        <v>20</v>
-      </c>
-      <c r="N43" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A44" s="25" t="s">
-        <v>60</v>
-      </c>
-      <c r="B44" t="s">
-        <v>101</v>
-      </c>
-      <c r="D44" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="E44" t="s">
-        <v>20</v>
-      </c>
-      <c r="M44" t="s">
-        <v>20</v>
-      </c>
-      <c r="N44" t="s">
-        <v>20</v>
-      </c>
-      <c r="O44" s="9" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A45" s="25" t="s">
-        <v>61</v>
-      </c>
-      <c r="B45" t="s">
-        <v>62</v>
-      </c>
-      <c r="D45" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="F45" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="46" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="26" t="s">
-        <v>63</v>
-      </c>
-      <c r="B46" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="C46" s="7"/>
-      <c r="D46" s="8"/>
-      <c r="G46" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="H46" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="I46" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="J46" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="L46" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="M46" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="N46" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="O46" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
+      </c>
+    </row>
+    <row r="44" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="26" t="s">
+        <v>105</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C44" s="7"/>
+      <c r="D44" s="8"/>
+      <c r="G44" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="H44" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="I44" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="J44" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="L44" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="M44" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="N44" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="O44" s="7" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Marsch am ende raus
</commit_message>
<xml_diff>
--- a/besetzung.xlsx
+++ b/besetzung.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Thadden27\thadden27\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git\thadden27\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B74584BE-AB6F-4E64-88D7-6F6F27058D51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CF0D39D-5D34-4E0C-B484-DB3499A4EFC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{870A77A3-6497-424F-BFDB-56D4CBDBF5BF}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{870A77A3-6497-424F-BFDB-56D4CBDBF5BF}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="103">
   <si>
     <t>Szene</t>
   </si>
@@ -191,9 +191,6 @@
     <t>Multible Enden</t>
   </si>
   <si>
-    <t>Ermordung Elisabeth v. Thadden</t>
-  </si>
-  <si>
     <t xml:space="preserve">Dystopie </t>
   </si>
   <si>
@@ -305,9 +302,6 @@
     <t>Tanz um die Mitte</t>
   </si>
   <si>
-    <t>Mach End o Herr mach Ende</t>
-  </si>
-  <si>
     <t>Osterfeier</t>
   </si>
   <si>
@@ -335,25 +329,22 @@
     <t>11.3</t>
   </si>
   <si>
-    <t>12a.1</t>
-  </si>
-  <si>
-    <t>12a.2</t>
-  </si>
-  <si>
-    <t>12b.1</t>
-  </si>
-  <si>
-    <t>12b.2</t>
-  </si>
-  <si>
-    <t>12c</t>
-  </si>
-  <si>
-    <t>12d</t>
-  </si>
-  <si>
     <t>13</t>
+  </si>
+  <si>
+    <t>Ermordung Elisabeth "Mach End o Herr"</t>
+  </si>
+  <si>
+    <t>12.1</t>
+  </si>
+  <si>
+    <t>12.2</t>
+  </si>
+  <si>
+    <t>12.3</t>
+  </si>
+  <si>
+    <t>12.4</t>
   </si>
 </sst>
 </file>
@@ -477,7 +468,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="16" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
@@ -513,6 +504,7 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -869,24 +861,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7EAA9A49-82B2-433C-BF39-5078DFD427BF}">
-  <dimension ref="A1:O44"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:O42"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.5703125" style="25"/>
-    <col min="2" max="2" width="40.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.85546875" style="9" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.5546875" style="25"/>
+    <col min="2" max="2" width="40.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.88671875" style="9" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="6" style="10" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.140625" style="9" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.140625" style="10" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="19.5703125" style="9" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.5546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.109375" style="9" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.109375" style="10" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="19.5546875" style="9" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A1" s="25" t="s">
         <v>0</v>
       </c>
@@ -900,13 +892,13 @@
         <v>25</v>
       </c>
       <c r="E1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F1" t="s">
         <v>30</v>
       </c>
       <c r="G1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="H1" s="5" t="s">
         <v>2</v>
@@ -933,12 +925,12 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="26" t="s">
         <v>10</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C2" s="7" t="s">
         <v>19</v>
@@ -948,7 +940,7 @@
       <c r="J2" s="8"/>
       <c r="O2" s="7"/>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3" s="25" t="s">
         <v>11</v>
       </c>
@@ -959,13 +951,13 @@
         <v>19</v>
       </c>
       <c r="G3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="N3" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4" s="25" t="s">
         <v>15</v>
       </c>
@@ -979,7 +971,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5" s="25" t="s">
         <v>16</v>
       </c>
@@ -990,7 +982,7 @@
         <v>19</v>
       </c>
       <c r="G5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="J5" s="10" t="s">
         <v>19</v>
@@ -999,7 +991,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6" s="25" t="s">
         <v>17</v>
       </c>
@@ -1010,7 +1002,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="7" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A7" s="26" t="s">
         <v>20</v>
       </c>
@@ -1026,7 +1018,7 @@
       <c r="E7" s="2"/>
       <c r="F7" s="2"/>
       <c r="G7" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="H7" s="7"/>
       <c r="J7" s="8"/>
@@ -1035,7 +1027,7 @@
       </c>
       <c r="O7" s="7"/>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8" s="25" t="s">
         <v>48</v>
       </c>
@@ -1051,7 +1043,7 @@
       <c r="E8" s="21"/>
       <c r="F8" s="21"/>
       <c r="G8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="H8" s="9" t="s">
         <v>19</v>
@@ -1072,7 +1064,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:15" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" s="26" t="s">
         <v>22</v>
       </c>
@@ -1090,7 +1082,7 @@
       <c r="J9" s="17"/>
       <c r="O9" s="16"/>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10" s="25" t="s">
         <v>26</v>
       </c>
@@ -1101,15 +1093,15 @@
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11" s="25" t="s">
         <v>27</v>
       </c>
       <c r="B11" s="24" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G11" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="H11" s="9" t="s">
         <v>19</v>
@@ -1127,12 +1119,12 @@
         <v>19</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12" s="25" t="s">
         <v>29</v>
       </c>
       <c r="B12" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F12" t="s">
         <v>19</v>
@@ -1141,12 +1133,12 @@
         <v>19</v>
       </c>
     </row>
-    <row r="13" spans="1:15" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:15" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A13" s="26" t="s">
         <v>31</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C13" s="16" t="s">
         <v>19</v>
@@ -1159,69 +1151,69 @@
       <c r="J13" s="17"/>
       <c r="O13" s="16"/>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14" s="25" t="s">
+        <v>69</v>
+      </c>
+      <c r="B14" t="s">
+        <v>71</v>
+      </c>
+      <c r="C14" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="G14" t="s">
+        <v>60</v>
+      </c>
+      <c r="H14" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="I14" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A15" s="25" t="s">
         <v>70</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B15" t="s">
+        <v>74</v>
+      </c>
+      <c r="C15" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="F15" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A16" s="25" t="s">
         <v>72</v>
       </c>
-      <c r="C14" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="G14" t="s">
-        <v>61</v>
-      </c>
-      <c r="H14" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="I14" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A15" s="25" t="s">
-        <v>71</v>
-      </c>
-      <c r="B15" t="s">
+      <c r="B16" t="s">
+        <v>73</v>
+      </c>
+      <c r="C16" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="G16" t="s">
+        <v>60</v>
+      </c>
+      <c r="H16" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="I16" t="s">
+        <v>19</v>
+      </c>
+      <c r="O16" s="9" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="26" t="s">
+        <v>55</v>
+      </c>
+      <c r="B17" s="1" t="s">
         <v>75</v>
-      </c>
-      <c r="C15" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="F15" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A16" s="25" t="s">
-        <v>73</v>
-      </c>
-      <c r="B16" t="s">
-        <v>74</v>
-      </c>
-      <c r="C16" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="G16" t="s">
-        <v>61</v>
-      </c>
-      <c r="H16" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="I16" t="s">
-        <v>19</v>
-      </c>
-      <c r="O16" s="9" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="17" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="26" t="s">
-        <v>56</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>76</v>
       </c>
       <c r="C17" s="7"/>
       <c r="D17" s="8" t="s">
@@ -1234,12 +1226,12 @@
       <c r="J17" s="8"/>
       <c r="O17" s="7"/>
     </row>
-    <row r="18" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A18" s="26" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C18" s="7" t="s">
         <v>19</v>
@@ -1249,9 +1241,9 @@
       <c r="J18" s="8"/>
       <c r="O18" s="7"/>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A19" s="25" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B19" t="s">
         <v>34</v>
@@ -1263,12 +1255,12 @@
         <v>19</v>
       </c>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A20" s="25" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B20" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C20" s="9" t="s">
         <v>19</v>
@@ -1277,7 +1269,7 @@
         <v>19</v>
       </c>
       <c r="G20" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="L20" t="s">
         <v>19</v>
@@ -1289,7 +1281,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="21" spans="1:15" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:15" s="18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A21" s="27" t="s">
         <v>36</v>
       </c>
@@ -1299,7 +1291,7 @@
       <c r="J21" s="20"/>
       <c r="O21" s="19"/>
     </row>
-    <row r="22" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A22" s="26" t="s">
         <v>32</v>
       </c>
@@ -1314,7 +1306,7 @@
       <c r="J22" s="8"/>
       <c r="O22" s="7"/>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A23" s="25" t="s">
         <v>33</v>
       </c>
@@ -1328,7 +1320,7 @@
         <v>19</v>
       </c>
       <c r="G23" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="M23" t="s">
         <v>19</v>
@@ -1337,7 +1329,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A24" s="25" t="s">
         <v>35</v>
       </c>
@@ -1351,7 +1343,7 @@
         <v>19</v>
       </c>
       <c r="G24" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="I24" t="s">
         <v>19</v>
@@ -1366,9 +1358,9 @@
         <v>19</v>
       </c>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A25" s="25" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B25" t="s">
         <v>42</v>
@@ -1380,7 +1372,7 @@
         <v>19</v>
       </c>
       <c r="G25" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="K25" t="s">
         <v>19</v>
@@ -1389,9 +1381,9 @@
         <v>19</v>
       </c>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A26" s="25" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B26" t="s">
         <v>43</v>
@@ -1403,7 +1395,7 @@
         <v>19</v>
       </c>
       <c r="G26" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="I26" t="s">
         <v>19</v>
@@ -1415,12 +1407,12 @@
         <v>19</v>
       </c>
     </row>
-    <row r="27" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A27" s="26" t="s">
         <v>37</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C27" s="7" t="s">
         <v>19</v>
@@ -1433,12 +1425,12 @@
       <c r="J27" s="8"/>
       <c r="O27" s="7"/>
     </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A28" s="25" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B28" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C28" s="9" t="s">
         <v>19</v>
@@ -1450,12 +1442,12 @@
         <v>19</v>
       </c>
     </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A29" s="25" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B29" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C29" s="9" t="s">
         <v>19</v>
@@ -1464,12 +1456,12 @@
         <v>19</v>
       </c>
     </row>
-    <row r="30" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A30" s="26" t="s">
         <v>44</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C30" s="7"/>
       <c r="D30" s="8" t="s">
@@ -1479,12 +1471,12 @@
       <c r="J30" s="8"/>
       <c r="O30" s="7"/>
     </row>
-    <row r="31" spans="1:15" s="28" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:15" s="28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A31" s="25" t="s">
         <v>39</v>
       </c>
       <c r="B31" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C31" s="29"/>
       <c r="D31" s="30" t="s">
@@ -1494,7 +1486,7 @@
         <v>19</v>
       </c>
       <c r="G31" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="H31" s="29"/>
       <c r="J31" s="30" t="s">
@@ -1505,12 +1497,12 @@
       </c>
       <c r="O31" s="29"/>
     </row>
-    <row r="32" spans="1:15" s="32" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:15" s="32" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A32" s="31" t="s">
         <v>45</v>
       </c>
       <c r="B32" s="32" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C32" s="33" t="s">
         <v>19</v>
@@ -1523,12 +1515,12 @@
       <c r="J32" s="34"/>
       <c r="O32" s="33"/>
     </row>
-    <row r="33" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A33" s="26" t="s">
         <v>46</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C33" s="7"/>
       <c r="D33" s="8" t="s">
@@ -1538,26 +1530,26 @@
       <c r="J33" s="8"/>
       <c r="O33" s="7"/>
     </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A34" s="25" t="s">
+        <v>82</v>
+      </c>
+      <c r="B34" t="s">
+        <v>81</v>
+      </c>
+      <c r="D34" s="10" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="35" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A35" s="25" t="s">
         <v>83</v>
       </c>
-      <c r="B34" t="s">
-        <v>82</v>
-      </c>
-      <c r="D34" s="10" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A35" s="25" t="s">
-        <v>84</v>
-      </c>
       <c r="B35" s="24" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G35" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="H35" s="9" t="s">
         <v>19</v>
@@ -1575,12 +1567,12 @@
         <v>19</v>
       </c>
     </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A36" s="25" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B36" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D36" s="10" t="s">
         <v>19</v>
@@ -1598,7 +1590,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="37" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A37" s="26" t="s">
         <v>47</v>
       </c>
@@ -1615,12 +1607,12 @@
       <c r="J37" s="8"/>
       <c r="O37" s="7"/>
     </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A38" s="25" t="s">
         <v>99</v>
       </c>
       <c r="B38" t="s">
-        <v>51</v>
+        <v>98</v>
       </c>
       <c r="C38" s="9" t="s">
         <v>19</v>
@@ -1628,47 +1620,62 @@
       <c r="F38" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="G38" t="s">
+        <v>58</v>
+      </c>
+      <c r="H38" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="I38" s="35" t="s">
+        <v>19</v>
+      </c>
+      <c r="J38" s="10" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="39" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A39" s="25" t="s">
         <v>100</v>
       </c>
       <c r="B39" t="s">
-        <v>89</v>
-      </c>
-      <c r="G39" t="s">
-        <v>59</v>
-      </c>
-      <c r="H39" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="I39" t="s">
-        <v>19</v>
-      </c>
-      <c r="J39" s="10" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.25">
+        <v>51</v>
+      </c>
+      <c r="D39" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="F39" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="40" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A40" s="25" t="s">
         <v>101</v>
       </c>
       <c r="B40" t="s">
-        <v>52</v>
+        <v>87</v>
       </c>
       <c r="D40" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="F40" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="E40" t="s">
+        <v>19</v>
+      </c>
+      <c r="M40" t="s">
+        <v>19</v>
+      </c>
+      <c r="N40" t="s">
+        <v>19</v>
+      </c>
+      <c r="O40" s="9" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="41" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A41" s="25" t="s">
         <v>102</v>
       </c>
       <c r="B41" t="s">
-        <v>18</v>
+        <v>52</v>
       </c>
       <c r="D41" s="10" t="s">
         <v>19</v>
@@ -1676,87 +1683,38 @@
       <c r="F41" t="s">
         <v>19</v>
       </c>
-      <c r="G41" t="s">
-        <v>63</v>
-      </c>
-      <c r="L41" t="s">
-        <v>19</v>
-      </c>
-      <c r="M41" t="s">
-        <v>19</v>
-      </c>
-      <c r="N41" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A42" s="25" t="s">
-        <v>103</v>
-      </c>
-      <c r="B42" t="s">
-        <v>88</v>
-      </c>
-      <c r="D42" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="E42" t="s">
-        <v>19</v>
-      </c>
-      <c r="M42" t="s">
-        <v>19</v>
-      </c>
-      <c r="N42" t="s">
-        <v>19</v>
-      </c>
-      <c r="O42" s="9" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A43" s="25" t="s">
-        <v>104</v>
-      </c>
-      <c r="B43" t="s">
+    </row>
+    <row r="42" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="26" t="s">
+        <v>97</v>
+      </c>
+      <c r="B42" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="D43" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="F43" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="44" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="26" t="s">
-        <v>105</v>
-      </c>
-      <c r="B44" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="C44" s="7"/>
-      <c r="D44" s="8"/>
-      <c r="G44" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="H44" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="I44" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="J44" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="L44" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="M44" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="N44" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="O44" s="7" t="s">
+      <c r="C42" s="7"/>
+      <c r="D42" s="8"/>
+      <c r="G42" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="H42" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="I42" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="J42" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="L42" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="M42" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="N42" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="O42" s="7" t="s">
         <v>19</v>
       </c>
     </row>

</xml_diff>